<commit_message>
PROVA - cambiata logica ritardi su indicazioni dottorandi
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_input/Estrazione 8/vettori.xlsx
+++ b/PS-VRP/Dati_input/Estrazione 8/vettori.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frenc\Documents\GitHub\progettoIS\PS-VRP\Dati_input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Frenc\Documents\GitHub\progettoIS\PS-VRP\Dati_input\Estrazione 8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC77B75E-71BA-4D9F-934D-41D9F6367DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFDF765D-7823-4BF4-91A7-A6054FDD8208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9135" yWindow="2490" windowWidth="16665" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yyyy"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -75,19 +75,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -102,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -111,6 +117,19 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -461,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="22.28515625" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -521,14 +540,57 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>40032</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>45848</v>
       </c>
-      <c r="D5" s="2">
+      <c r="C5" s="6"/>
+      <c r="D5" s="4">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>240025</v>
+      </c>
+      <c r="B6" s="8">
+        <v>45848</v>
+      </c>
+      <c r="C6" s="7">
+        <v>4</v>
+      </c>
+      <c r="D6" s="7">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>240003</v>
+      </c>
+      <c r="B7" s="8">
+        <v>45849</v>
+      </c>
+      <c r="C7" s="7">
+        <v>11</v>
+      </c>
+      <c r="D7" s="7">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>240046</v>
+      </c>
+      <c r="B8" s="8">
+        <v>45850</v>
+      </c>
+      <c r="C8" s="7">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7">
+        <v>14680</v>
       </c>
     </row>
   </sheetData>

</xml_diff>